<commit_message>
Base: operação em campanha
</commit_message>
<xml_diff>
--- a/00-esmagadora-modelo/dados_sujos/apontamentos_mensais/producao_2025_01.xlsx
+++ b/00-esmagadora-modelo/dados_sujos/apontamentos_mensais/producao_2025_01.xlsx
@@ -844,25 +844,25 @@
         <v>45672</v>
       </c>
       <c r="B19" t="n">
-        <v>1404.98</v>
+        <v>664.74</v>
       </c>
       <c r="C19" t="n">
-        <v>23.04</v>
+        <v>10.79</v>
       </c>
       <c r="D19" t="n">
-        <v>1027.14</v>
+        <v>477.79</v>
       </c>
       <c r="E19" t="n">
-        <v>276.36</v>
+        <v>132.18</v>
       </c>
       <c r="F19" t="n">
-        <v>2005</v>
+        <v>723</v>
       </c>
       <c r="G19" t="n">
-        <v>399795</v>
+        <v>184756</v>
       </c>
       <c r="H19" t="n">
-        <v>64395</v>
+        <v>30680</v>
       </c>
     </row>
     <row r="20">
@@ -870,25 +870,25 @@
         <v>45673</v>
       </c>
       <c r="B20" t="n">
-        <v>1481.3</v>
+        <v>1483.78</v>
       </c>
       <c r="C20" t="n">
         <v>24</v>
       </c>
       <c r="D20" t="n">
-        <v>1069.05</v>
+        <v>1084.08</v>
       </c>
       <c r="E20" t="n">
-        <v>300.78</v>
+        <v>303.98</v>
       </c>
       <c r="F20" t="n">
-        <v>2301</v>
+        <v>1199</v>
       </c>
       <c r="G20" t="n">
-        <v>402319</v>
+        <v>415574</v>
       </c>
       <c r="H20" t="n">
-        <v>68072</v>
+        <v>63652</v>
       </c>
     </row>
     <row r="21">
@@ -896,25 +896,25 @@
         <v>45674</v>
       </c>
       <c r="B21" t="n">
-        <v>1486.41</v>
+        <v>1447.29</v>
       </c>
       <c r="C21" t="n">
-        <v>24</v>
+        <v>23.53</v>
       </c>
       <c r="D21" t="n">
-        <v>1077.84</v>
+        <v>1045.56</v>
       </c>
       <c r="E21" t="n">
-        <v>302.11</v>
+        <v>299.37</v>
       </c>
       <c r="F21" t="n">
-        <v>2666</v>
+        <v>1158</v>
       </c>
       <c r="G21" t="n">
-        <v>400487</v>
+        <v>394109</v>
       </c>
       <c r="H21" t="n">
-        <v>63261</v>
+        <v>66153</v>
       </c>
     </row>
     <row r="22">
@@ -922,25 +922,25 @@
         <v>45675</v>
       </c>
       <c r="B22" t="n">
-        <v>1528.31</v>
+        <v>1468.82</v>
       </c>
       <c r="C22" t="n">
         <v>24</v>
       </c>
       <c r="D22" t="n">
-        <v>1106.03</v>
+        <v>1060.91</v>
       </c>
       <c r="E22" t="n">
-        <v>305.34</v>
+        <v>297.52</v>
       </c>
       <c r="F22" t="n">
-        <v>2273</v>
+        <v>1295</v>
       </c>
       <c r="G22" t="n">
-        <v>400078</v>
+        <v>443318</v>
       </c>
       <c r="H22" t="n">
-        <v>69468</v>
+        <v>68504</v>
       </c>
     </row>
     <row r="23">
@@ -948,25 +948,25 @@
         <v>45676</v>
       </c>
       <c r="B23" t="n">
-        <v>1389.7</v>
+        <v>1393.38</v>
       </c>
       <c r="C23" t="n">
-        <v>21.66</v>
+        <v>24</v>
       </c>
       <c r="D23" t="n">
-        <v>1010.39</v>
+        <v>1005.5</v>
       </c>
       <c r="E23" t="n">
-        <v>286.07</v>
+        <v>287.04</v>
       </c>
       <c r="F23" t="n">
-        <v>1924</v>
+        <v>1298</v>
       </c>
       <c r="G23" t="n">
-        <v>373349</v>
+        <v>361125</v>
       </c>
       <c r="H23" t="n">
-        <v>61206</v>
+        <v>61004</v>
       </c>
     </row>
     <row r="24">
@@ -974,25 +974,25 @@
         <v>45677</v>
       </c>
       <c r="B24" t="n">
-        <v>1366.32</v>
+        <v>1404.55</v>
       </c>
       <c r="C24" t="n">
-        <v>24</v>
+        <v>23.37</v>
       </c>
       <c r="D24" t="n">
-        <v>992.14</v>
+        <v>1020.75</v>
       </c>
       <c r="E24" t="n">
-        <v>268.41</v>
+        <v>284.05</v>
       </c>
       <c r="F24" t="n">
-        <v>2092</v>
+        <v>1511</v>
       </c>
       <c r="G24" t="n">
-        <v>343171</v>
+        <v>370592</v>
       </c>
       <c r="H24" t="n">
-        <v>62948</v>
+        <v>63107</v>
       </c>
     </row>
     <row r="25">
@@ -1000,25 +1000,25 @@
         <v>45678</v>
       </c>
       <c r="B25" t="n">
-        <v>1479.28</v>
+        <v>1478.5</v>
       </c>
       <c r="C25" t="n">
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>1068.46</v>
+        <v>1072.28</v>
       </c>
       <c r="E25" t="n">
-        <v>290.8</v>
+        <v>294.05</v>
       </c>
       <c r="F25" t="n">
-        <v>2143</v>
+        <v>1715</v>
       </c>
       <c r="G25" t="n">
-        <v>386790</v>
+        <v>384326</v>
       </c>
       <c r="H25" t="n">
-        <v>70345</v>
+        <v>67365</v>
       </c>
     </row>
     <row r="26">
@@ -1026,25 +1026,25 @@
         <v>45679</v>
       </c>
       <c r="B26" t="n">
-        <v>1522.23</v>
+        <v>1477.4</v>
       </c>
       <c r="C26" t="n">
         <v>24</v>
       </c>
       <c r="D26" t="n">
-        <v>1108.22</v>
+        <v>1066.98</v>
       </c>
       <c r="E26" t="n">
-        <v>280.86</v>
+        <v>302.81</v>
       </c>
       <c r="F26" t="n">
-        <v>1800</v>
+        <v>1320</v>
       </c>
       <c r="G26" t="n">
-        <v>416382</v>
+        <v>398508</v>
       </c>
       <c r="H26" t="n">
-        <v>67381</v>
+        <v>62043</v>
       </c>
     </row>
     <row r="27">
@@ -1052,25 +1052,25 @@
         <v>45680</v>
       </c>
       <c r="B27" t="n">
-        <v>1240.02</v>
+        <v>1465.38</v>
       </c>
       <c r="C27" t="n">
-        <v>20.53</v>
+        <v>22.88</v>
       </c>
       <c r="D27" t="n">
-        <v>891.29</v>
+        <v>1060.95</v>
       </c>
       <c r="E27" t="n">
-        <v>250.14</v>
+        <v>291.49</v>
       </c>
       <c r="F27" t="n">
-        <v>1799</v>
+        <v>1248</v>
       </c>
       <c r="G27" t="n">
-        <v>297564</v>
+        <v>401018</v>
       </c>
       <c r="H27" t="n">
-        <v>53783</v>
+        <v>69433</v>
       </c>
     </row>
     <row r="28">
@@ -1078,25 +1078,25 @@
         <v>45681</v>
       </c>
       <c r="B28" t="n">
-        <v>1414.62</v>
+        <v>1515.34</v>
       </c>
       <c r="C28" t="n">
-        <v>22.73</v>
+        <v>24</v>
       </c>
       <c r="D28" t="n">
-        <v>1019.13</v>
+        <v>1084.76</v>
       </c>
       <c r="E28" t="n">
-        <v>282.84</v>
+        <v>303.66</v>
       </c>
       <c r="F28" t="n">
-        <v>1921</v>
+        <v>1573</v>
       </c>
       <c r="G28" t="n">
-        <v>381129</v>
+        <v>380076</v>
       </c>
       <c r="H28" t="n">
-        <v>62424</v>
+        <v>64830</v>
       </c>
     </row>
     <row r="29">
@@ -1104,25 +1104,25 @@
         <v>45682</v>
       </c>
       <c r="B29" t="n">
-        <v>1360.47</v>
+        <v>1504.96</v>
       </c>
       <c r="C29" t="n">
         <v>24</v>
       </c>
       <c r="D29" t="n">
-        <v>991.83</v>
+        <v>1090.2</v>
       </c>
       <c r="E29" t="n">
-        <v>265.55</v>
+        <v>290.52</v>
       </c>
       <c r="F29" t="n">
-        <v>2334</v>
+        <v>1433</v>
       </c>
       <c r="G29" t="n">
-        <v>372959</v>
+        <v>396627</v>
       </c>
       <c r="H29" t="n">
-        <v>63787</v>
+        <v>63867</v>
       </c>
     </row>
     <row r="30">
@@ -1130,25 +1130,25 @@
         <v>45683</v>
       </c>
       <c r="B30" t="n">
-        <v>1495.9</v>
+        <v>1303.26</v>
       </c>
       <c r="C30" t="n">
-        <v>24</v>
+        <v>23.6</v>
       </c>
       <c r="D30" t="n">
-        <v>1088.6</v>
+        <v>939.6900000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>295.73</v>
+        <v>263.04</v>
       </c>
       <c r="F30" t="n">
-        <v>2153</v>
+        <v>1336</v>
       </c>
       <c r="G30" t="n">
-        <v>412407</v>
+        <v>395694</v>
       </c>
       <c r="H30" t="n">
-        <v>68581</v>
+        <v>63117</v>
       </c>
     </row>
     <row r="31">
@@ -1156,25 +1156,25 @@
         <v>45684</v>
       </c>
       <c r="B31" t="n">
-        <v>1535.13</v>
+        <v>1507.17</v>
       </c>
       <c r="C31" t="n">
-        <v>23.84</v>
+        <v>23.71</v>
       </c>
       <c r="D31" t="n">
-        <v>1112.36</v>
+        <v>1084.65</v>
       </c>
       <c r="E31" t="n">
-        <v>308.15</v>
+        <v>300.51</v>
       </c>
       <c r="F31" t="n">
-        <v>2090</v>
+        <v>1131</v>
       </c>
       <c r="G31" t="n">
-        <v>419963</v>
+        <v>416813</v>
       </c>
       <c r="H31" t="n">
-        <v>65564</v>
+        <v>64560</v>
       </c>
     </row>
     <row r="32">
@@ -1182,25 +1182,25 @@
         <v>45685</v>
       </c>
       <c r="B32" t="n">
-        <v>519.35</v>
+        <v>530.4299999999999</v>
       </c>
       <c r="C32" t="n">
         <v>8.77</v>
       </c>
       <c r="D32" t="n">
-        <v>376.22</v>
+        <v>384.52</v>
       </c>
       <c r="E32" t="n">
-        <v>104.44</v>
+        <v>105.04</v>
       </c>
       <c r="F32" t="n">
-        <v>1036</v>
+        <v>778</v>
       </c>
       <c r="G32" t="n">
-        <v>150730</v>
+        <v>154294</v>
       </c>
       <c r="H32" t="n">
-        <v>23063</v>
+        <v>23185</v>
       </c>
     </row>
     <row r="33">
@@ -1208,25 +1208,25 @@
         <v>45686</v>
       </c>
       <c r="B33" t="n">
-        <v>1558.67</v>
+        <v>1478.54</v>
       </c>
       <c r="C33" t="n">
         <v>24</v>
       </c>
       <c r="D33" t="n">
-        <v>1133.77</v>
+        <v>1068.48</v>
       </c>
       <c r="E33" t="n">
-        <v>314.72</v>
+        <v>295.1</v>
       </c>
       <c r="F33" t="n">
-        <v>2486</v>
+        <v>1228</v>
       </c>
       <c r="G33" t="n">
-        <v>409973</v>
+        <v>399863</v>
       </c>
       <c r="H33" t="n">
-        <v>69664</v>
+        <v>63922</v>
       </c>
     </row>
     <row r="34">
@@ -1234,25 +1234,25 @@
         <v>45687</v>
       </c>
       <c r="B34" t="n">
-        <v>1540.75</v>
+        <v>1468.61</v>
       </c>
       <c r="C34" t="n">
         <v>24</v>
       </c>
       <c r="D34" t="n">
-        <v>1118.08</v>
+        <v>1057.37</v>
       </c>
       <c r="E34" t="n">
-        <v>314.05</v>
+        <v>286.88</v>
       </c>
       <c r="F34" t="n">
-        <v>2214</v>
+        <v>1400</v>
       </c>
       <c r="G34" t="n">
-        <v>412991</v>
+        <v>359668</v>
       </c>
       <c r="H34" t="n">
-        <v>68903</v>
+        <v>67769</v>
       </c>
     </row>
     <row r="35">
@@ -1260,25 +1260,25 @@
         <v>45688</v>
       </c>
       <c r="B35" t="n">
-        <v>1280.35</v>
+        <v>1491.99</v>
       </c>
       <c r="C35" t="n">
-        <v>21.83</v>
+        <v>23.78</v>
       </c>
       <c r="D35" t="n">
-        <v>919.75</v>
+        <v>1077.48</v>
       </c>
       <c r="E35" t="n">
-        <v>253.06</v>
+        <v>292.12</v>
       </c>
       <c r="F35" t="n">
-        <v>1693</v>
+        <v>1376</v>
       </c>
       <c r="G35" t="n">
-        <v>372447</v>
+        <v>437791</v>
       </c>
       <c r="H35" t="n">
-        <v>63185</v>
+        <v>67020</v>
       </c>
     </row>
     <row r="37">
@@ -1288,25 +1288,25 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>23603.79</v>
+        <v>23084.14</v>
       </c>
       <c r="C37" t="n">
-        <v>382.4</v>
+        <v>376.4299999999999</v>
       </c>
       <c r="D37" t="n">
-        <v>17110.3</v>
+        <v>16681.95</v>
       </c>
       <c r="E37" t="n">
-        <v>4699.410000000001</v>
+        <v>4629.36</v>
       </c>
       <c r="F37" t="n">
-        <v>34930</v>
+        <v>21722</v>
       </c>
       <c r="G37" t="n">
-        <v>6352534</v>
+        <v>6294152</v>
       </c>
       <c r="H37" t="n">
-        <v>1066030</v>
+        <v>1030211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustando base de dados para estudo.
</commit_message>
<xml_diff>
--- a/00-esmagadora-modelo/dados_sujos/apontamentos_mensais/producao_2025_01.xlsx
+++ b/00-esmagadora-modelo/dados_sujos/apontamentos_mensais/producao_2025_01.xlsx
@@ -844,25 +844,25 @@
         <v>45672</v>
       </c>
       <c r="B19" t="n">
-        <v>664.74</v>
+        <v>731.62</v>
       </c>
       <c r="C19" t="n">
-        <v>10.79</v>
+        <v>12.2</v>
       </c>
       <c r="D19" t="n">
-        <v>477.79</v>
+        <v>530.9400000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>132.18</v>
+        <v>148.95</v>
       </c>
       <c r="F19" t="n">
-        <v>723</v>
+        <v>755</v>
       </c>
       <c r="G19" t="n">
-        <v>184756</v>
+        <v>216692</v>
       </c>
       <c r="H19" t="n">
-        <v>30680</v>
+        <v>32237</v>
       </c>
     </row>
     <row r="20">
@@ -870,25 +870,25 @@
         <v>45673</v>
       </c>
       <c r="B20" t="n">
-        <v>1483.78</v>
+        <v>1474.14</v>
       </c>
       <c r="C20" t="n">
         <v>24</v>
       </c>
       <c r="D20" t="n">
-        <v>1084.08</v>
+        <v>1078.27</v>
       </c>
       <c r="E20" t="n">
-        <v>303.98</v>
+        <v>294.7</v>
       </c>
       <c r="F20" t="n">
-        <v>1199</v>
+        <v>1156</v>
       </c>
       <c r="G20" t="n">
-        <v>415574</v>
+        <v>399390</v>
       </c>
       <c r="H20" t="n">
-        <v>63652</v>
+        <v>67264</v>
       </c>
     </row>
     <row r="21">
@@ -896,25 +896,25 @@
         <v>45674</v>
       </c>
       <c r="B21" t="n">
-        <v>1447.29</v>
+        <v>1469.62</v>
       </c>
       <c r="C21" t="n">
-        <v>23.53</v>
+        <v>24</v>
       </c>
       <c r="D21" t="n">
-        <v>1045.56</v>
+        <v>1055.72</v>
       </c>
       <c r="E21" t="n">
-        <v>299.37</v>
+        <v>291.1</v>
       </c>
       <c r="F21" t="n">
-        <v>1158</v>
+        <v>1527</v>
       </c>
       <c r="G21" t="n">
-        <v>394109</v>
+        <v>430686</v>
       </c>
       <c r="H21" t="n">
-        <v>66153</v>
+        <v>70965</v>
       </c>
     </row>
     <row r="22">
@@ -922,25 +922,25 @@
         <v>45675</v>
       </c>
       <c r="B22" t="n">
-        <v>1468.82</v>
+        <v>1531.47</v>
       </c>
       <c r="C22" t="n">
         <v>24</v>
       </c>
       <c r="D22" t="n">
-        <v>1060.91</v>
+        <v>1105.77</v>
       </c>
       <c r="E22" t="n">
-        <v>297.52</v>
+        <v>303.01</v>
       </c>
       <c r="F22" t="n">
-        <v>1295</v>
+        <v>1378</v>
       </c>
       <c r="G22" t="n">
-        <v>443318</v>
+        <v>370287</v>
       </c>
       <c r="H22" t="n">
-        <v>68504</v>
+        <v>70209</v>
       </c>
     </row>
     <row r="23">
@@ -948,25 +948,25 @@
         <v>45676</v>
       </c>
       <c r="B23" t="n">
-        <v>1393.38</v>
+        <v>1421.23</v>
       </c>
       <c r="C23" t="n">
         <v>24</v>
       </c>
       <c r="D23" t="n">
-        <v>1005.5</v>
+        <v>1017.63</v>
       </c>
       <c r="E23" t="n">
-        <v>287.04</v>
+        <v>278.27</v>
       </c>
       <c r="F23" t="n">
-        <v>1298</v>
+        <v>1225</v>
       </c>
       <c r="G23" t="n">
-        <v>361125</v>
+        <v>397429</v>
       </c>
       <c r="H23" t="n">
-        <v>61004</v>
+        <v>61711</v>
       </c>
     </row>
     <row r="24">
@@ -974,25 +974,25 @@
         <v>45677</v>
       </c>
       <c r="B24" t="n">
-        <v>1404.55</v>
+        <v>1490.38</v>
       </c>
       <c r="C24" t="n">
-        <v>23.37</v>
+        <v>24</v>
       </c>
       <c r="D24" t="n">
-        <v>1020.75</v>
+        <v>1082.25</v>
       </c>
       <c r="E24" t="n">
-        <v>284.05</v>
+        <v>293.49</v>
       </c>
       <c r="F24" t="n">
-        <v>1511</v>
+        <v>1642</v>
       </c>
       <c r="G24" t="n">
-        <v>370592</v>
+        <v>379724</v>
       </c>
       <c r="H24" t="n">
-        <v>63107</v>
+        <v>66470</v>
       </c>
     </row>
     <row r="25">
@@ -1000,25 +1000,25 @@
         <v>45678</v>
       </c>
       <c r="B25" t="n">
-        <v>1478.5</v>
+        <v>1543.59</v>
       </c>
       <c r="C25" t="n">
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>1072.28</v>
+        <v>1128.06</v>
       </c>
       <c r="E25" t="n">
-        <v>294.05</v>
+        <v>314.58</v>
       </c>
       <c r="F25" t="n">
-        <v>1715</v>
+        <v>1640</v>
       </c>
       <c r="G25" t="n">
-        <v>384326</v>
+        <v>406232</v>
       </c>
       <c r="H25" t="n">
-        <v>67365</v>
+        <v>68186</v>
       </c>
     </row>
     <row r="26">
@@ -1026,25 +1026,25 @@
         <v>45679</v>
       </c>
       <c r="B26" t="n">
-        <v>1477.4</v>
+        <v>1396.58</v>
       </c>
       <c r="C26" t="n">
         <v>24</v>
       </c>
       <c r="D26" t="n">
-        <v>1066.98</v>
+        <v>1010.34</v>
       </c>
       <c r="E26" t="n">
-        <v>302.81</v>
+        <v>273.25</v>
       </c>
       <c r="F26" t="n">
-        <v>1320</v>
+        <v>1184</v>
       </c>
       <c r="G26" t="n">
-        <v>398508</v>
+        <v>367801</v>
       </c>
       <c r="H26" t="n">
-        <v>62043</v>
+        <v>63409</v>
       </c>
     </row>
     <row r="27">
@@ -1052,25 +1052,25 @@
         <v>45680</v>
       </c>
       <c r="B27" t="n">
-        <v>1465.38</v>
+        <v>1265.41</v>
       </c>
       <c r="C27" t="n">
-        <v>22.88</v>
+        <v>19.71</v>
       </c>
       <c r="D27" t="n">
-        <v>1060.95</v>
+        <v>915.47</v>
       </c>
       <c r="E27" t="n">
-        <v>291.49</v>
+        <v>243.18</v>
       </c>
       <c r="F27" t="n">
-        <v>1248</v>
+        <v>1548</v>
       </c>
       <c r="G27" t="n">
-        <v>401018</v>
+        <v>343212</v>
       </c>
       <c r="H27" t="n">
-        <v>69433</v>
+        <v>58838</v>
       </c>
     </row>
     <row r="28">
@@ -1078,25 +1078,25 @@
         <v>45681</v>
       </c>
       <c r="B28" t="n">
-        <v>1515.34</v>
+        <v>1465.88</v>
       </c>
       <c r="C28" t="n">
-        <v>24</v>
+        <v>23.66</v>
       </c>
       <c r="D28" t="n">
-        <v>1084.76</v>
+        <v>1068.54</v>
       </c>
       <c r="E28" t="n">
-        <v>303.66</v>
+        <v>294.05</v>
       </c>
       <c r="F28" t="n">
-        <v>1573</v>
+        <v>1222</v>
       </c>
       <c r="G28" t="n">
-        <v>380076</v>
+        <v>391159</v>
       </c>
       <c r="H28" t="n">
-        <v>64830</v>
+        <v>64542</v>
       </c>
     </row>
     <row r="29">
@@ -1104,25 +1104,25 @@
         <v>45682</v>
       </c>
       <c r="B29" t="n">
-        <v>1504.96</v>
+        <v>1567.17</v>
       </c>
       <c r="C29" t="n">
-        <v>24</v>
+        <v>23.39</v>
       </c>
       <c r="D29" t="n">
-        <v>1090.2</v>
+        <v>1129.22</v>
       </c>
       <c r="E29" t="n">
-        <v>290.52</v>
+        <v>314.84</v>
       </c>
       <c r="F29" t="n">
-        <v>1433</v>
+        <v>1450</v>
       </c>
       <c r="G29" t="n">
-        <v>396627</v>
+        <v>409826</v>
       </c>
       <c r="H29" t="n">
-        <v>63867</v>
+        <v>68978</v>
       </c>
     </row>
     <row r="30">
@@ -1130,25 +1130,25 @@
         <v>45683</v>
       </c>
       <c r="B30" t="n">
-        <v>1303.26</v>
+        <v>1484.03</v>
       </c>
       <c r="C30" t="n">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="D30" t="n">
-        <v>939.6900000000001</v>
+        <v>1074.46</v>
       </c>
       <c r="E30" t="n">
-        <v>263.04</v>
+        <v>301.98</v>
       </c>
       <c r="F30" t="n">
-        <v>1336</v>
+        <v>1412</v>
       </c>
       <c r="G30" t="n">
-        <v>395694</v>
+        <v>362659</v>
       </c>
       <c r="H30" t="n">
-        <v>63117</v>
+        <v>63899</v>
       </c>
     </row>
     <row r="31">
@@ -1156,25 +1156,25 @@
         <v>45684</v>
       </c>
       <c r="B31" t="n">
-        <v>1507.17</v>
+        <v>1439.03</v>
       </c>
       <c r="C31" t="n">
-        <v>23.71</v>
+        <v>23.33</v>
       </c>
       <c r="D31" t="n">
-        <v>1084.65</v>
+        <v>1037.75</v>
       </c>
       <c r="E31" t="n">
-        <v>300.51</v>
+        <v>288.36</v>
       </c>
       <c r="F31" t="n">
-        <v>1131</v>
+        <v>1438</v>
       </c>
       <c r="G31" t="n">
-        <v>416813</v>
+        <v>378489</v>
       </c>
       <c r="H31" t="n">
-        <v>64560</v>
+        <v>66574</v>
       </c>
     </row>
     <row r="32">
@@ -1182,25 +1182,25 @@
         <v>45685</v>
       </c>
       <c r="B32" t="n">
-        <v>530.4299999999999</v>
+        <v>565.67</v>
       </c>
       <c r="C32" t="n">
         <v>8.77</v>
       </c>
       <c r="D32" t="n">
-        <v>384.52</v>
+        <v>411.01</v>
       </c>
       <c r="E32" t="n">
-        <v>105.04</v>
+        <v>109.77</v>
       </c>
       <c r="F32" t="n">
-        <v>778</v>
+        <v>479</v>
       </c>
       <c r="G32" t="n">
-        <v>154294</v>
+        <v>159466</v>
       </c>
       <c r="H32" t="n">
-        <v>23185</v>
+        <v>25175</v>
       </c>
     </row>
     <row r="33">
@@ -1208,25 +1208,25 @@
         <v>45686</v>
       </c>
       <c r="B33" t="n">
-        <v>1478.54</v>
+        <v>1511.47</v>
       </c>
       <c r="C33" t="n">
         <v>24</v>
       </c>
       <c r="D33" t="n">
-        <v>1068.48</v>
+        <v>1088.64</v>
       </c>
       <c r="E33" t="n">
-        <v>295.1</v>
+        <v>307.14</v>
       </c>
       <c r="F33" t="n">
-        <v>1228</v>
+        <v>1203</v>
       </c>
       <c r="G33" t="n">
-        <v>399863</v>
+        <v>408884</v>
       </c>
       <c r="H33" t="n">
-        <v>63922</v>
+        <v>66914</v>
       </c>
     </row>
     <row r="34">
@@ -1234,25 +1234,25 @@
         <v>45687</v>
       </c>
       <c r="B34" t="n">
-        <v>1468.61</v>
+        <v>1396.25</v>
       </c>
       <c r="C34" t="n">
         <v>24</v>
       </c>
       <c r="D34" t="n">
-        <v>1057.37</v>
+        <v>1017.54</v>
       </c>
       <c r="E34" t="n">
-        <v>286.88</v>
+        <v>279.16</v>
       </c>
       <c r="F34" t="n">
-        <v>1400</v>
+        <v>983</v>
       </c>
       <c r="G34" t="n">
-        <v>359668</v>
+        <v>388069</v>
       </c>
       <c r="H34" t="n">
-        <v>67769</v>
+        <v>62742</v>
       </c>
     </row>
     <row r="35">
@@ -1260,25 +1260,25 @@
         <v>45688</v>
       </c>
       <c r="B35" t="n">
-        <v>1491.99</v>
+        <v>1306.88</v>
       </c>
       <c r="C35" t="n">
-        <v>23.78</v>
+        <v>21.06</v>
       </c>
       <c r="D35" t="n">
-        <v>1077.48</v>
+        <v>939.41</v>
       </c>
       <c r="E35" t="n">
-        <v>292.12</v>
+        <v>256.23</v>
       </c>
       <c r="F35" t="n">
-        <v>1376</v>
+        <v>1257</v>
       </c>
       <c r="G35" t="n">
-        <v>437791</v>
+        <v>327164</v>
       </c>
       <c r="H35" t="n">
-        <v>67020</v>
+        <v>56609</v>
       </c>
     </row>
     <row r="37">
@@ -1288,25 +1288,25 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>23084.14</v>
+        <v>23060.42</v>
       </c>
       <c r="C37" t="n">
-        <v>376.4299999999999</v>
+        <v>372.1199999999999</v>
       </c>
       <c r="D37" t="n">
-        <v>16681.95</v>
+        <v>16691.02</v>
       </c>
       <c r="E37" t="n">
-        <v>4629.36</v>
+        <v>4592.059999999999</v>
       </c>
       <c r="F37" t="n">
-        <v>21722</v>
+        <v>21499</v>
       </c>
       <c r="G37" t="n">
-        <v>6294152</v>
+        <v>6137169</v>
       </c>
       <c r="H37" t="n">
-        <v>1030211</v>
+        <v>1034722</v>
       </c>
     </row>
   </sheetData>

</xml_diff>